<commit_message>
10/22 manu revision. redo table s1
</commit_message>
<xml_diff>
--- a/fire nutrient/raw_data/fire history/excel fire histories.xlsx
+++ b/fire nutrient/raw_data/fire history/excel fire histories.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\VFT\VFT_github\zyao78VFTcode\Legacy effect\raw-data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\PhD\VFT\VFT_github\zyao78VFTcode\fire nutrient\raw_data\fire history\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{394BDC25-3893-4E14-8C95-8D838C56C18D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0E5EB90-49C8-4624-B0B3-CD446A90D7D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="45960" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{58B67793-E89C-414F-A104-ABAD252BA177}"/>
+    <workbookView xWindow="45960" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="3" xr2:uid="{58B67793-E89C-414F-A104-ABAD252BA177}"/>
   </bookViews>
   <sheets>
     <sheet name="manager" sheetId="1" r:id="rId1"/>
@@ -254,10 +254,6 @@
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
   <si>
-    <t xml:space="preserve">We determine a landscape fire has occurred when: 1) Manager fire history is backed up by Landsat (not necessarily the exact population pixel but the general landscape). </t>
-    <phoneticPr fontId="5" type="noConversion"/>
-  </si>
-  <si>
     <t>startyear</t>
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
@@ -280,6 +276,9 @@
   <si>
     <t>ME</t>
     <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">We determine a landscape fire has occurred when: 1) Manager fire history is backed up by Landsat (not necessarily the exact population pixel but the general landscape). </t>
   </si>
 </sst>
 </file>
@@ -3094,21 +3093,16 @@
       <c r="A1" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="H1" s="2" t="s">
-        <v>65</v>
-      </c>
     </row>
     <row r="2" spans="1:24">
       <c r="A2" s="5" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B2" s="5" t="s">
         <v>2</v>
       </c>
       <c r="C2" s="5"/>
-      <c r="M2" s="2" t="s">
-        <v>67</v>
-      </c>
+      <c r="M2" s="2"/>
       <c r="N2" s="2"/>
       <c r="O2" s="2"/>
       <c r="P2" s="2"/>
@@ -3144,6 +3138,9 @@
       <c r="B5" t="s">
         <v>17</v>
       </c>
+      <c r="M5" t="s">
+        <v>71</v>
+      </c>
     </row>
     <row r="6" spans="1:24">
       <c r="A6">
@@ -3152,6 +3149,9 @@
       <c r="B6" t="s">
         <v>17</v>
       </c>
+      <c r="R6" s="2" t="s">
+        <v>66</v>
+      </c>
     </row>
     <row r="7" spans="1:24">
       <c r="A7">
@@ -3334,7 +3334,7 @@
         <v>2006</v>
       </c>
       <c r="B29" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="30" spans="1:2">
@@ -3342,7 +3342,7 @@
         <v>2009</v>
       </c>
       <c r="B30" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="31" spans="1:2">
@@ -3350,7 +3350,7 @@
         <v>2020</v>
       </c>
       <c r="B31" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="32" spans="1:2">
@@ -3358,7 +3358,7 @@
         <v>2008</v>
       </c>
       <c r="B32" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="33" spans="1:2">
@@ -3366,7 +3366,7 @@
         <v>2011</v>
       </c>
       <c r="B33" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="34" spans="1:2">
@@ -3374,7 +3374,7 @@
         <v>2015</v>
       </c>
       <c r="B34" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="35" spans="1:2">
@@ -3382,7 +3382,7 @@
         <v>2017</v>
       </c>
       <c r="B35" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="36" spans="1:2">
@@ -3390,7 +3390,7 @@
         <v>2019</v>
       </c>
       <c r="B36" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="37" spans="1:2">
@@ -3398,7 +3398,7 @@
         <v>2021</v>
       </c>
       <c r="B37" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="38" spans="1:2">
@@ -3406,7 +3406,7 @@
         <v>2011</v>
       </c>
       <c r="B38" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="39" spans="1:2">
@@ -3414,7 +3414,7 @@
         <v>2014</v>
       </c>
       <c r="B39" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="40" spans="1:2">
@@ -3422,7 +3422,7 @@
         <v>2019</v>
       </c>
       <c r="B40" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="41" spans="1:2">
@@ -3430,7 +3430,7 @@
         <v>2022</v>
       </c>
       <c r="B41" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="42" spans="1:2">
@@ -3438,7 +3438,7 @@
         <v>2008</v>
       </c>
       <c r="B42" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="43" spans="1:2">
@@ -3446,7 +3446,7 @@
         <v>2011</v>
       </c>
       <c r="B43" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="44" spans="1:2">
@@ -3454,7 +3454,7 @@
         <v>2014</v>
       </c>
       <c r="B44" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="45" spans="1:2">
@@ -3462,7 +3462,7 @@
         <v>2016</v>
       </c>
       <c r="B45" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="46" spans="1:2">
@@ -3470,7 +3470,7 @@
         <v>2019</v>
       </c>
       <c r="B46" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
   </sheetData>

</xml_diff>